<commit_message>
fixed gross profit not being processed properly, added categories to removed index, changed token trigger from financials to financial
</commit_message>
<xml_diff>
--- a/categories_index_removed.xlsx
+++ b/categories_index_removed.xlsx
@@ -4,44 +4,55 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" tabRatio="600" autoFilterDateGrouping="true"/>
   </bookViews>
   <sheets>
-    <sheet name="cash_bank" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="accounts_receivable" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="fixed_assets" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="depreciation_amortization" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="accounts_payable" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="credit_cards" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="payroll_liabilities" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="payroll_benefits" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="deferred_revenue" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="equity" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="loans_liabilities" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="accrued_liabilities" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="income_revenue" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="cogs" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="advertising_marketing" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="auto_expenses" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="bank_fees" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="meals_entertainment" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="travel" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="office_supplies" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="repairs_maintenance" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="taxes_licenses" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="interest_expense" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="bonuses_commissions" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="consulting_legal_it" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="general_expenses" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="misc" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="cash_bank" sheetId="1" r:id="rId1" state="visible"/>
+    <sheet name="accounts_receivable" sheetId="2" r:id="rId2" state="visible"/>
+    <sheet name="fixed_assets" sheetId="3" r:id="rId3" state="visible"/>
+    <sheet name="depreciation_amortization" sheetId="4" r:id="rId4" state="visible"/>
+    <sheet name="accounts_payable" sheetId="5" r:id="rId5" state="visible"/>
+    <sheet name="credit_cards" sheetId="6" r:id="rId6" state="visible"/>
+    <sheet name="payroll_liabilities" sheetId="7" r:id="rId7" state="visible"/>
+    <sheet name="payroll_benefits" sheetId="8" r:id="rId8" state="visible"/>
+    <sheet name="deferred_revenue" sheetId="9" r:id="rId9" state="visible"/>
+    <sheet name="equity" sheetId="10" r:id="rId10" state="visible"/>
+    <sheet name="loans_liabilities" sheetId="11" r:id="rId11" state="visible"/>
+    <sheet name="accrued_liabilities" sheetId="12" r:id="rId12" state="visible"/>
+    <sheet name="income_revenue" sheetId="13" r:id="rId13" state="visible"/>
+    <sheet name="cogs" sheetId="14" r:id="rId14" state="visible"/>
+    <sheet name="advertising_marketing" sheetId="15" r:id="rId15" state="visible"/>
+    <sheet name="auto_expenses" sheetId="16" r:id="rId16" state="visible"/>
+    <sheet name="bank_fees" sheetId="17" r:id="rId17" state="visible"/>
+    <sheet name="meals_entertainment" sheetId="18" r:id="rId18" state="visible"/>
+    <sheet name="travel" sheetId="19" r:id="rId19" state="visible"/>
+    <sheet name="office_supplies" sheetId="20" r:id="rId20" state="visible"/>
+    <sheet name="repairs_maintenance" sheetId="21" r:id="rId21" state="visible"/>
+    <sheet name="taxes_licenses" sheetId="22" r:id="rId22" state="visible"/>
+    <sheet name="interest_expense" sheetId="23" r:id="rId23" state="visible"/>
+    <sheet name="bonuses_commissions" sheetId="24" r:id="rId24" state="visible"/>
+    <sheet name="consulting_legal_it" sheetId="25" r:id="rId25" state="visible"/>
+    <sheet name="general_expenses" sheetId="26" r:id="rId26" state="visible"/>
+    <sheet name="misc" sheetId="27" r:id="rId27" state="visible"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="true"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+  <si>
+    <t>6024 Employee Reimbursement</t>
+  </si>
+  <si>
+    <t>7001 Cash Reward</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <numFmts count="0"/>
   <fonts count="2">
     <font>
@@ -82,13 +93,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="false" pivotButton="false"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" quotePrefix="false" pivotButton="false"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="false"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium9"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -161,7 +172,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -13123,15 +13134,15 @@
 </file>
 
 <file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="true" summaryRight="true"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="55" customWidth="1" min="1" max="1"/>
+    <col customWidth="true" max="1" min="1" width="55"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13833,6 +13844,11 @@
         <is>
           <t>8800 Other Miscellaneous Expense</t>
         </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="s">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -19205,15 +19221,15 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="true" summaryRight="true"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="55" customWidth="1" min="1" max="1"/>
+    <col customWidth="true" max="1" min="1" width="55"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -20370,6 +20386,11 @@
         <is>
           <t>7004 Credit Card Rewards</t>
         </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="s">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>